<commit_message>
need to update how system adds duplicate parts (recursive functions still not working)
</commit_message>
<xml_diff>
--- a/shipClassTests/AuxilaryPropulsionPlant_Reliability_Availability_Data.xlsx
+++ b/shipClassTests/AuxilaryPropulsionPlant_Reliability_Availability_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adware\Desktop\KISS\shipClassTests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7904F7CB-4882-4B86-8729-AB0F78D3C706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DC0A4A1-92CD-458D-8E2C-9D01940BA431}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="195" windowWidth="19200" windowHeight="11085" firstSheet="1" activeTab="1" xr2:uid="{279480E9-DBDF-4252-B432-4CE1D30BF378}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{279480E9-DBDF-4252-B432-4CE1D30BF378}"/>
   </bookViews>
   <sheets>
     <sheet name="machinery reliability data" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="32">
   <si>
     <t>Component</t>
   </si>
@@ -121,13 +121,19 @@
     <t>[8, 9, 10, 11, 12, 6, 0, 1]</t>
   </si>
   <si>
-    <t>[]</t>
-  </si>
-  <si>
     <t xml:space="preserve">diesel engine #1 system </t>
   </si>
   <si>
     <t xml:space="preserve">diesel engine #2 system </t>
+  </si>
+  <si>
+    <t xml:space="preserve">fuel system </t>
+  </si>
+  <si>
+    <t>[(2,3)]</t>
+  </si>
+  <si>
+    <t>[([5,6], [5,6]), (7,7)]</t>
   </si>
 </sst>
 </file>
@@ -536,15 +542,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F997A0B-9C86-4EC5-9A0F-10545207BFB0}">
   <dimension ref="A1:F37"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.73046875" customWidth="1"/>
-    <col min="2" max="2" width="24.1328125" customWidth="1"/>
-    <col min="3" max="3" width="18.265625" style="2" customWidth="1"/>
-    <col min="4" max="6" width="18.265625" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="24.140625" customWidth="1"/>
+    <col min="3" max="3" width="18.28515625" style="2" customWidth="1"/>
+    <col min="4" max="6" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>20</v>
       </c>
@@ -564,7 +570,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
@@ -584,7 +590,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -604,7 +610,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -624,7 +630,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -644,7 +650,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -664,7 +670,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -684,7 +690,7 @@
         <v>0.997</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -704,7 +710,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -724,7 +730,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -744,7 +750,7 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -764,7 +770,7 @@
         <v>0.998</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -784,7 +790,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -804,7 +810,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -824,7 +830,7 @@
         <v>0.999</v>
       </c>
     </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.45">
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C37" s="5"/>
     </row>
   </sheetData>
@@ -836,12 +842,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD4FF0A7-4C32-4212-8D10-DADC32F7B7B8}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="3" width="32.3984375" customWidth="1"/>
+    <col min="2" max="3" width="32.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>22</v>
       </c>
@@ -852,40 +858,51 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2</v>
       </c>
       <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
         <v>23</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D6" s="4"/>
     </row>
   </sheetData>
@@ -897,21 +914,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B338D18E-1C2C-4003-BC79-5462DE0704E2}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.1328125" customWidth="1"/>
-    <col min="2" max="2" width="30.3984375" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
+    <col min="2" max="2" width="30.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B1" s="1"/>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>